<commit_message>
📊 BIST Screener | 23.04.2026 08:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-23.xlsx
+++ b/data/bist_screener_2026-04-23.xlsx
@@ -25781,52 +25781,50 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>6.13</v>
+        <v>81.84</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0.0016</v>
+        <v>0.0027</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>8730000</v>
+        <v>11800000</v>
       </c>
       <c r="E583" s="6" t="inlineStr"/>
       <c r="F583" s="7" t="n">
-        <v>61.01</v>
+        <v>45.85</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
       <c r="I583" s="6" t="inlineStr"/>
       <c r="J583" s="6" t="inlineStr"/>
-      <c r="K583" s="6" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
+      <c r="K583" s="6" t="inlineStr"/>
       <c r="L583" s="6" t="inlineStr"/>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>197.4</v>
+        <v>251</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.099</v>
+        <v>-0.0346</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>20610000</v>
-      </c>
-      <c r="E584" s="2" t="inlineStr"/>
+        <v>8590</v>
+      </c>
+      <c r="E584" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F584" s="3" t="n">
-        <v>45.87</v>
+        <v>46.72</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
@@ -25834,36 +25832,30 @@
       <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L584" s="2" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L584" s="2" t="inlineStr"/>
       <c r="M584" s="2" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>251</v>
+        <v>169</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>-0.0346</v>
+        <v>0.0236</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>8590</v>
-      </c>
-      <c r="E585" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>12070000</v>
+      </c>
+      <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>46.72</v>
+        <v>60.59</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
@@ -25871,31 +25863,33 @@
       <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L585" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L585" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+        </is>
+      </c>
       <c r="M585" s="6" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>16.08</v>
+        <v>18.99</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.0111</v>
+        <v>-0.0495</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>72700000</v>
+        <v>102290000</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
-      <c r="F586" s="3" t="n">
-        <v>51.02</v>
-      </c>
+      <c r="F586" s="2" t="inlineStr"/>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
       <c r="I586" s="2" t="inlineStr"/>
@@ -25907,7 +25901,7 @@
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25915,106 +25909,110 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>4.73</v>
+        <v>80.95</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0216</v>
+        <v>0.0247</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>62450000</v>
+        <v>32400</v>
       </c>
       <c r="E587" s="8" t="n">
-        <v>0.8667</v>
+        <v>0.58</v>
       </c>
       <c r="F587" s="7" t="n">
-        <v>77.90000000000001</v>
+        <v>41.16</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="6" t="inlineStr"/>
-      <c r="J587" s="6" t="inlineStr"/>
+      <c r="I587" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J587" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr"/>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>80.95</v>
+        <v>197.4</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0247</v>
+        <v>-0.099</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>32400</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>20610000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>41.16</v>
+        <v>45.87</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J588" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I588" s="2" t="inlineStr"/>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>18.99</v>
+        <v>62.95</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0495</v>
+        <v>-0.0008</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>102290000</v>
-      </c>
-      <c r="E589" s="6" t="inlineStr"/>
-      <c r="F589" s="6" t="inlineStr"/>
+        <v>539710</v>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
+      <c r="F589" s="7" t="n">
+        <v>56.09</v>
+      </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
       <c r="I589" s="6" t="inlineStr"/>
-      <c r="J589" s="6" t="inlineStr"/>
+      <c r="J589" s="8" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26022,34 +26020,38 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>2.82</v>
+        <v>10.56</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0537</v>
+        <v>0.08529999999999999</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>263430000</v>
-      </c>
-      <c r="E590" s="2" t="inlineStr"/>
+        <v>255670000</v>
+      </c>
+      <c r="E590" s="4" t="n">
+        <v>0.2479</v>
+      </c>
       <c r="F590" s="3" t="n">
-        <v>52.07</v>
+        <v>53.86</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="2" t="inlineStr"/>
+      <c r="I590" s="4" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26057,40 +26059,34 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>2.74</v>
+        <v>13.89</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0108</v>
+        <v>0.0102</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>98340000</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>35540000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>43.27</v>
+        <v>54.23</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J591" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I591" s="6" t="inlineStr"/>
+      <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26133,122 +26129,124 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>24.62</v>
+        <v>7.59</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.004099999999999999</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>15600000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>477650</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>56.05</v>
+        <v>39.58</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J593" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>81.84</v>
+        <v>24.62</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0027</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>11800000</v>
+        <v>15600000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>45.85</v>
+        <v>56.05</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
       <c r="I594" s="2" t="inlineStr"/>
       <c r="J594" s="2" t="inlineStr"/>
-      <c r="K594" s="2" t="inlineStr"/>
-      <c r="L594" s="2" t="inlineStr"/>
+      <c r="K594" s="2" t="inlineStr">
+        <is>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>62.95</v>
+        <v>103.5</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0008</v>
+        <v>-0.001</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>539710</v>
-      </c>
-      <c r="E595" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
-      <c r="F595" s="7" t="n">
-        <v>56.09</v>
-      </c>
+        <v>398550</v>
+      </c>
+      <c r="E595" s="6" t="inlineStr"/>
+      <c r="F595" s="6" t="inlineStr"/>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="8" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr"/>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>13.89</v>
+        <v>4.73</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0102</v>
+        <v>0.0216</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>35540000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>62450000</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>54.23</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26256,12 +26254,12 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26269,21 +26267,21 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>39.64</v>
+        <v>2.82</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0195</v>
+        <v>-0.0537</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>12770000</v>
+        <v>263430000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>52.02</v>
+        <v>52.07</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26291,12 +26289,12 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26304,38 +26302,40 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>10.56</v>
+        <v>2.74</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.08529999999999999</v>
+        <v>-0.0108</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>255670000</v>
+        <v>98340000</v>
       </c>
       <c r="E598" s="4" t="n">
-        <v>0.2479</v>
+        <v>0.7119</v>
       </c>
       <c r="F598" s="3" t="n">
-        <v>53.86</v>
+        <v>43.27</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="4" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
-      <c r="J598" s="2" t="inlineStr"/>
+        <v>-191.6342</v>
+      </c>
+      <c r="J598" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26343,21 +26343,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>33.9</v>
+        <v>16.08</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0174</v>
+        <v>-0.0111</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>4590000</v>
+        <v>72700000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>54.07</v>
+        <v>51.02</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26365,12 +26365,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26378,42 +26378,40 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>17.32</v>
+        <v>152.1</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0058</v>
+        <v>-0.0225</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>12210000</v>
+        <v>2330000</v>
       </c>
       <c r="E600" s="4" t="n">
-        <v>0.9246</v>
+        <v>0.1071</v>
       </c>
       <c r="F600" s="3" t="n">
-        <v>47.99</v>
-      </c>
-      <c r="G600" s="3" t="n">
-        <v>163.71</v>
-      </c>
+        <v>52.17</v>
+      </c>
+      <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="4" t="n">
-        <v>0.0028</v>
+        <v>-3.6635</v>
       </c>
       <c r="J600" s="4" t="n">
-        <v>-10.3171</v>
+        <v>-0.4897</v>
       </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26421,110 +26419,108 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>6.95</v>
+        <v>6.13</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.09970000000000001</v>
+        <v>0.0016</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>75580000</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>8730000</v>
+      </c>
+      <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>78.58</v>
+        <v>61.01</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
         </is>
       </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>103.5</v>
+        <v>28.66</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.001</v>
+        <v>-0.0478</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>398550</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
-      <c r="F602" s="2" t="inlineStr"/>
+        <v>18930000</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.2667</v>
+      </c>
+      <c r="F602" s="3" t="n">
+        <v>50.42</v>
+      </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>152.1</v>
+        <v>6.95</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0225</v>
+        <v>-0.09970000000000001</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>2330000</v>
+        <v>75580000</v>
       </c>
       <c r="E603" s="8" t="n">
-        <v>0.1071</v>
+        <v>0.1672</v>
       </c>
       <c r="F603" s="7" t="n">
-        <v>52.17</v>
+        <v>78.58</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
       <c r="I603" s="8" t="n">
-        <v>-3.6635</v>
+        <v>-5.3262</v>
       </c>
       <c r="J603" s="8" t="n">
-        <v>-0.4897</v>
+        <v>-4.2562</v>
       </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26532,21 +26528,21 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>90.84999999999999</v>
+        <v>33.9</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0595</v>
+        <v>-0.0174</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>14880000</v>
+        <v>4590000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>61.35</v>
+        <v>54.07</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26554,12 +26550,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26567,21 +26563,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>169</v>
+        <v>39.64</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0236</v>
+        <v>0.0195</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>12070000</v>
+        <v>12770000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>60.59</v>
+        <v>52.02</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26589,7 +26585,7 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
@@ -26602,36 +26598,42 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>28.66</v>
+        <v>17.32</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0478</v>
+        <v>0.0058</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>18930000</v>
+        <v>12210000</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.2667</v>
+        <v>0.9246</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>50.42</v>
-      </c>
-      <c r="G606" s="2" t="inlineStr"/>
+        <v>47.99</v>
+      </c>
+      <c r="G606" s="3" t="n">
+        <v>163.71</v>
+      </c>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="2" t="inlineStr"/>
+      <c r="I606" s="4" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J606" s="4" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26639,38 +26641,36 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>7.59</v>
+        <v>90.84999999999999</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.007800000000000001</v>
+        <v>-0.0595</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>477650</v>
-      </c>
-      <c r="E607" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>14880000</v>
+      </c>
+      <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>39.58</v>
+        <v>61.35</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J607" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I607" s="6" t="inlineStr"/>
+      <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26695,7 +26695,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>23.04.2026 07:30</t>
+          <t>23.04.2026 08:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 23.04.2026 09:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-23.xlsx
+++ b/data/bist_screener_2026-04-23.xlsx
@@ -25781,94 +25781,116 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>81.84</v>
+        <v>39.64</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0.0027</v>
+        <v>0.0195</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>11800000</v>
+        <v>12770000</v>
       </c>
       <c r="E583" s="6" t="inlineStr"/>
       <c r="F583" s="7" t="n">
-        <v>45.85</v>
+        <v>52.02</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
       <c r="I583" s="6" t="inlineStr"/>
       <c r="J583" s="6" t="inlineStr"/>
-      <c r="K583" s="6" t="inlineStr"/>
-      <c r="L583" s="6" t="inlineStr"/>
+      <c r="K583" s="6" t="inlineStr">
+        <is>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+        </is>
+      </c>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>251</v>
+        <v>2.74</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0346</v>
+        <v>-0.0108</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>8590</v>
+        <v>98340000</v>
       </c>
       <c r="E584" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.7119</v>
       </c>
       <c r="F584" s="3" t="n">
-        <v>46.72</v>
+        <v>43.27</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
-      <c r="I584" s="2" t="inlineStr"/>
-      <c r="J584" s="2" t="inlineStr"/>
+      <c r="I584" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J584" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L584" s="2" t="inlineStr"/>
+          <t>Dağıtım servisleri</t>
+        </is>
+      </c>
+      <c r="L584" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M584" s="2" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>169</v>
+        <v>6.95</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.0236</v>
+        <v>-0.09970000000000001</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>12070000</v>
-      </c>
-      <c r="E585" s="6" t="inlineStr"/>
+        <v>75580000</v>
+      </c>
+      <c r="E585" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F585" s="7" t="n">
-        <v>60.59</v>
+        <v>78.58</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
-      <c r="I585" s="6" t="inlineStr"/>
-      <c r="J585" s="6" t="inlineStr"/>
+      <c r="I585" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J585" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25876,32 +25898,40 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>18.99</v>
+        <v>152.1</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.0495</v>
+        <v>-0.0225</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>102290000</v>
-      </c>
-      <c r="E586" s="2" t="inlineStr"/>
-      <c r="F586" s="2" t="inlineStr"/>
+        <v>2330000</v>
+      </c>
+      <c r="E586" s="4" t="n">
+        <v>0.1071</v>
+      </c>
+      <c r="F586" s="3" t="n">
+        <v>52.17</v>
+      </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
-      <c r="I586" s="2" t="inlineStr"/>
-      <c r="J586" s="2" t="inlineStr"/>
+      <c r="I586" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J586" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25909,58 +25939,58 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>80.95</v>
+        <v>4.73</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0247</v>
+        <v>0.0216</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>32400</v>
+        <v>62450000</v>
       </c>
       <c r="E587" s="8" t="n">
-        <v>0.58</v>
+        <v>0.8667</v>
       </c>
       <c r="F587" s="7" t="n">
-        <v>41.16</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J587" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I587" s="6" t="inlineStr"/>
+      <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>197.4</v>
+        <v>16.08</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.099</v>
+        <v>-0.0111</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>20610000</v>
+        <v>72700000</v>
       </c>
       <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>45.87</v>
+        <v>51.02</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25968,12 +25998,12 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -26020,60 +26050,58 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>10.56</v>
+        <v>7.59</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.08529999999999999</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>255670000</v>
+        <v>477650</v>
       </c>
       <c r="E590" s="4" t="n">
-        <v>0.2479</v>
+        <v>0.95</v>
       </c>
       <c r="F590" s="3" t="n">
-        <v>53.86</v>
+        <v>39.58</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="4" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
-      <c r="J590" s="2" t="inlineStr"/>
+        <v>-23.6291</v>
+      </c>
+      <c r="J590" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr"/>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>13.89</v>
+        <v>41.38</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0102</v>
+        <v>0.0222</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>35540000</v>
+        <v>10990000</v>
       </c>
       <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>54.23</v>
+        <v>60.95</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26081,12 +26109,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26094,21 +26122,21 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>41.38</v>
+        <v>197.4</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0222</v>
+        <v>-0.099</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>10990000</v>
+        <v>20610000</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>60.95</v>
+        <v>45.87</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26116,12 +26144,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26129,38 +26157,36 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>7.59</v>
+        <v>169</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.007800000000000001</v>
+        <v>0.0236</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>477650</v>
-      </c>
-      <c r="E593" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>12070000</v>
+      </c>
+      <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>39.58</v>
+        <v>60.59</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J593" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I593" s="6" t="inlineStr"/>
+      <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
@@ -26201,52 +26227,56 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>103.5</v>
+        <v>90.84999999999999</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.001</v>
+        <v>-0.0595</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>398550</v>
+        <v>14880000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
-      <c r="F595" s="6" t="inlineStr"/>
+      <c r="F595" s="7" t="n">
+        <v>61.35</v>
+      </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>4.73</v>
+        <v>2.82</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0216</v>
+        <v>-0.0537</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>62450000</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>263430000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>77.90000000000001</v>
+        <v>52.07</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26259,7 +26289,7 @@
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26267,34 +26297,38 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>2.82</v>
+        <v>10.56</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0537</v>
+        <v>0.08529999999999999</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>263430000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>255670000</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.2479</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>52.07</v>
+        <v>53.86</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26302,62 +26336,48 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>2.74</v>
+        <v>81.84</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0108</v>
+        <v>0.0027</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>98340000</v>
-      </c>
-      <c r="E598" s="4" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>11800000</v>
+      </c>
+      <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>43.27</v>
+        <v>45.85</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J598" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
-      <c r="K598" s="2" t="inlineStr">
-        <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+      <c r="I598" s="2" t="inlineStr"/>
+      <c r="J598" s="2" t="inlineStr"/>
+      <c r="K598" s="2" t="inlineStr"/>
+      <c r="L598" s="2" t="inlineStr"/>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>16.08</v>
+        <v>13.89</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0111</v>
+        <v>0.0102</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>72700000</v>
+        <v>35540000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>51.02</v>
+        <v>54.23</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26365,12 +26385,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26378,40 +26398,34 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>152.1</v>
+        <v>33.9</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0225</v>
+        <v>-0.0174</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>2330000</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>4590000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>52.17</v>
+        <v>54.07</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26419,22 +26433,20 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>6.13</v>
+        <v>18.99</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0016</v>
+        <v>-0.0495</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>8730000</v>
+        <v>102290000</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
-      <c r="F601" s="7" t="n">
-        <v>61.01</v>
-      </c>
+      <c r="F601" s="6" t="inlineStr"/>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
@@ -26444,42 +26456,52 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L601" s="6" t="inlineStr"/>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>28.66</v>
+        <v>17.32</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0478</v>
+        <v>0.0058</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>18930000</v>
+        <v>12210000</v>
       </c>
       <c r="E602" s="4" t="n">
-        <v>0.2667</v>
+        <v>0.9246</v>
       </c>
       <c r="F602" s="3" t="n">
-        <v>50.42</v>
-      </c>
-      <c r="G602" s="2" t="inlineStr"/>
+        <v>47.99</v>
+      </c>
+      <c r="G602" s="3" t="n">
+        <v>163.71</v>
+      </c>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="2" t="inlineStr"/>
-      <c r="J602" s="2" t="inlineStr"/>
+      <c r="I602" s="4" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J602" s="4" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26487,40 +26509,36 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>6.95</v>
+        <v>28.66</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.09970000000000001</v>
+        <v>-0.0478</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>75580000</v>
+        <v>18930000</v>
       </c>
       <c r="E603" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.2667</v>
       </c>
       <c r="F603" s="7" t="n">
-        <v>78.58</v>
+        <v>50.42</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26528,21 +26546,23 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>33.9</v>
+        <v>251</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0174</v>
+        <v>-0.0346</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>4590000</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>8590</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>54.07</v>
+        <v>46.72</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26550,112 +26570,96 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr"/>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>39.64</v>
+        <v>103.5</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0195</v>
+        <v>-0.001</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>12770000</v>
+        <v>398550</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
-      <c r="F605" s="7" t="n">
-        <v>52.02</v>
-      </c>
+      <c r="F605" s="6" t="inlineStr"/>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="6" t="inlineStr"/>
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>17.32</v>
+        <v>80.95</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0058</v>
+        <v>0.0247</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>12210000</v>
+        <v>32400</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.9246</v>
+        <v>0.58</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>47.99</v>
-      </c>
-      <c r="G606" s="3" t="n">
-        <v>163.71</v>
-      </c>
+        <v>41.16</v>
+      </c>
+      <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
       <c r="I606" s="4" t="n">
-        <v>0.0028</v>
+        <v>-9.409700000000001</v>
       </c>
       <c r="J606" s="4" t="n">
-        <v>-10.3171</v>
+        <v>-4.155</v>
       </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>90.84999999999999</v>
+        <v>6.13</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0595</v>
+        <v>0.0016</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>14880000</v>
+        <v>8730000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>61.35</v>
+        <v>61.01</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26663,14 +26667,10 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr"/>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26695,7 +26695,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>23.04.2026 08:30</t>
+          <t>23.04.2026 09:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 23.04.2026 10:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-23.xlsx
+++ b/data/bist_screener_2026-04-23.xlsx
@@ -25781,75 +25781,77 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>39.64</v>
+        <v>7.59</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0.0195</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>12770000</v>
-      </c>
-      <c r="E583" s="6" t="inlineStr"/>
+        <v>477650</v>
+      </c>
+      <c r="E583" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F583" s="7" t="n">
-        <v>52.02</v>
+        <v>39.58</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
-      <c r="I583" s="6" t="inlineStr"/>
-      <c r="J583" s="6" t="inlineStr"/>
+      <c r="I583" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J583" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L583" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr"/>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>2.74</v>
+        <v>6.95</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0108</v>
+        <v>-0.09970000000000001</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>98340000</v>
+        <v>75580000</v>
       </c>
       <c r="E584" s="4" t="n">
-        <v>0.7119</v>
+        <v>0.1672</v>
       </c>
       <c r="F584" s="3" t="n">
-        <v>43.27</v>
+        <v>78.58</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
       <c r="I584" s="4" t="n">
-        <v>-191.6342</v>
+        <v>-5.3262</v>
       </c>
       <c r="J584" s="4" t="n">
-        <v>-0.8093</v>
+        <v>-4.2562</v>
       </c>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25857,40 +25859,38 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>6.95</v>
+        <v>62.95</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>-0.09970000000000001</v>
+        <v>-0.0008</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>75580000</v>
+        <v>539710</v>
       </c>
       <c r="E585" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F585" s="7" t="n">
-        <v>78.58</v>
+        <v>56.09</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
-      <c r="I585" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
+      <c r="I585" s="6" t="inlineStr"/>
       <c r="J585" s="8" t="n">
-        <v>-4.2562</v>
+        <v>0.4139</v>
       </c>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25898,40 +25898,36 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>152.1</v>
+        <v>4.73</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.0225</v>
+        <v>0.0216</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>2330000</v>
+        <v>62450000</v>
       </c>
       <c r="E586" s="4" t="n">
-        <v>0.1071</v>
+        <v>0.8667</v>
       </c>
       <c r="F586" s="3" t="n">
-        <v>52.17</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
-      <c r="I586" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J586" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I586" s="2" t="inlineStr"/>
+      <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25939,23 +25935,21 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>4.73</v>
+        <v>169</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0216</v>
+        <v>0.0236</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>62450000</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>12070000</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>77.90000000000001</v>
+        <v>60.59</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25963,12 +25957,12 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25976,145 +25970,137 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>16.08</v>
+        <v>81.84</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0111</v>
+        <v>0.0027</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>72700000</v>
+        <v>11800000</v>
       </c>
       <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>51.02</v>
+        <v>45.85</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
       <c r="J588" s="2" t="inlineStr"/>
-      <c r="K588" s="2" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+      <c r="K588" s="2" t="inlineStr"/>
+      <c r="L588" s="2" t="inlineStr"/>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>62.95</v>
+        <v>80.95</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0008</v>
+        <v>0.0247</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>539710</v>
+        <v>32400</v>
       </c>
       <c r="E589" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.58</v>
       </c>
       <c r="F589" s="7" t="n">
-        <v>56.09</v>
+        <v>41.16</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="6" t="inlineStr"/>
+      <c r="I589" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
       <c r="J589" s="8" t="n">
-        <v>0.4139</v>
+        <v>-4.155</v>
       </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr"/>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>7.59</v>
+        <v>2.82</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.007800000000000001</v>
+        <v>-0.0537</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>477650</v>
-      </c>
-      <c r="E590" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>263430000</v>
+      </c>
+      <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>39.58</v>
+        <v>52.07</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J590" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I590" s="2" t="inlineStr"/>
+      <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>41.38</v>
+        <v>10.56</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0222</v>
+        <v>0.08529999999999999</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>10990000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>255670000</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.2479</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>60.95</v>
+        <v>53.86</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="6" t="inlineStr"/>
+      <c r="I591" s="8" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26122,21 +26108,23 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>197.4</v>
+        <v>28.66</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.099</v>
+        <v>-0.0478</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>20610000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>18930000</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>45.87</v>
+        <v>50.42</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26149,7 +26137,7 @@
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26157,21 +26145,23 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>169</v>
+        <v>251</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0236</v>
+        <v>-0.0346</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>12070000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>8590</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>60.59</v>
+        <v>46.72</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26179,34 +26169,30 @@
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>24.62</v>
+        <v>197.4</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.004099999999999999</v>
+        <v>-0.099</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>15600000</v>
+        <v>20610000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>56.05</v>
+        <v>45.87</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26214,12 +26200,12 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26227,21 +26213,21 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>90.84999999999999</v>
+        <v>41.38</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0595</v>
+        <v>0.0222</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>14880000</v>
+        <v>10990000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>61.35</v>
+        <v>60.95</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
@@ -26249,12 +26235,12 @@
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26262,21 +26248,21 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>2.82</v>
+        <v>33.9</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0537</v>
+        <v>-0.0174</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>263430000</v>
+        <v>4590000</v>
       </c>
       <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>52.07</v>
+        <v>54.07</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26284,12 +26270,12 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26297,38 +26283,42 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>10.56</v>
+        <v>17.32</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.08529999999999999</v>
+        <v>0.0058</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>255670000</v>
+        <v>12210000</v>
       </c>
       <c r="E597" s="8" t="n">
-        <v>0.2479</v>
+        <v>0.9246</v>
       </c>
       <c r="F597" s="7" t="n">
-        <v>53.86</v>
-      </c>
-      <c r="G597" s="6" t="inlineStr"/>
+        <v>47.99</v>
+      </c>
+      <c r="G597" s="7" t="n">
+        <v>163.71</v>
+      </c>
       <c r="H597" s="6" t="inlineStr"/>
       <c r="I597" s="8" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
-      <c r="J597" s="6" t="inlineStr"/>
+        <v>0.0028</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26336,48 +26326,56 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>81.84</v>
+        <v>90.84999999999999</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0027</v>
+        <v>-0.0595</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>11800000</v>
+        <v>14880000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>45.85</v>
+        <v>61.35</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
       <c r="J598" s="2" t="inlineStr"/>
-      <c r="K598" s="2" t="inlineStr"/>
-      <c r="L598" s="2" t="inlineStr"/>
+      <c r="K598" s="2" t="inlineStr">
+        <is>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>13.89</v>
+        <v>39.64</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0102</v>
+        <v>0.0195</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>35540000</v>
+        <v>12770000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>54.23</v>
+        <v>52.02</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26385,12 +26383,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26398,21 +26396,21 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>33.9</v>
+        <v>24.62</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0174</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>4590000</v>
+        <v>15600000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>54.07</v>
+        <v>56.05</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26420,12 +26418,12 @@
       <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26433,32 +26431,34 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>18.99</v>
+        <v>13.89</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0495</v>
+        <v>0.0102</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>102290000</v>
+        <v>35540000</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
-      <c r="F601" s="6" t="inlineStr"/>
+      <c r="F601" s="7" t="n">
+        <v>54.23</v>
+      </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26466,42 +26466,32 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>17.32</v>
+        <v>18.99</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0058</v>
+        <v>-0.0495</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>12210000</v>
-      </c>
-      <c r="E602" s="4" t="n">
-        <v>0.9246</v>
-      </c>
-      <c r="F602" s="3" t="n">
-        <v>47.99</v>
-      </c>
-      <c r="G602" s="3" t="n">
-        <v>163.71</v>
-      </c>
+        <v>102290000</v>
+      </c>
+      <c r="E602" s="2" t="inlineStr"/>
+      <c r="F602" s="2" t="inlineStr"/>
+      <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J602" s="4" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I602" s="2" t="inlineStr"/>
+      <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26509,36 +26499,40 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>28.66</v>
+        <v>2.74</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0478</v>
+        <v>-0.0108</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>18930000</v>
+        <v>98340000</v>
       </c>
       <c r="E603" s="8" t="n">
-        <v>0.2667</v>
+        <v>0.7119</v>
       </c>
       <c r="F603" s="7" t="n">
-        <v>50.42</v>
+        <v>43.27</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J603" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26546,31 +26540,27 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>251</v>
+        <v>103.5</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0346</v>
+        <v>-0.001</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>8590</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.2578</v>
-      </c>
-      <c r="F604" s="3" t="n">
-        <v>46.72</v>
-      </c>
+        <v>398550</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
+      <c r="F604" s="2" t="inlineStr"/>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="2" t="inlineStr"/>
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr"/>
@@ -26579,20 +26569,22 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>103.5</v>
+        <v>16.08</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.001</v>
+        <v>-0.0111</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>398550</v>
+        <v>72700000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
-      <c r="F605" s="6" t="inlineStr"/>
+      <c r="F605" s="7" t="n">
+        <v>51.02</v>
+      </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="6" t="inlineStr"/>
@@ -26602,41 +26594,39 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L605" s="6" t="inlineStr"/>
+      <c r="L605" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>80.95</v>
+        <v>6.13</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0247</v>
+        <v>0.0016</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>32400</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>8730000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>41.16</v>
+        <v>61.01</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J606" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr"/>
@@ -26645,32 +26635,42 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>6.13</v>
+        <v>152.1</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0016</v>
+        <v>-0.0225</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>8730000</v>
-      </c>
-      <c r="E607" s="6" t="inlineStr"/>
+        <v>2330000</v>
+      </c>
+      <c r="E607" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F607" s="7" t="n">
-        <v>61.01</v>
+        <v>52.17</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="6" t="inlineStr"/>
-      <c r="J607" s="6" t="inlineStr"/>
+      <c r="I607" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J607" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26695,7 +26695,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>23.04.2026 09:30</t>
+          <t>23.04.2026 10:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 23.04.2026 11:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-23.xlsx
+++ b/data/bist_screener_2026-04-23.xlsx
@@ -25781,77 +25781,67 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>7.59</v>
+        <v>18.99</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>-0.007800000000000001</v>
+        <v>-0.0495</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>477650</v>
-      </c>
-      <c r="E583" s="8" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F583" s="7" t="n">
-        <v>39.58</v>
-      </c>
+        <v>102290000</v>
+      </c>
+      <c r="E583" s="6" t="inlineStr"/>
+      <c r="F583" s="6" t="inlineStr"/>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
-      <c r="I583" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J583" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I583" s="6" t="inlineStr"/>
+      <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L583" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>6.95</v>
+        <v>169</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.09970000000000001</v>
+        <v>0.0236</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>75580000</v>
-      </c>
-      <c r="E584" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>12070000</v>
+      </c>
+      <c r="E584" s="2" t="inlineStr"/>
       <c r="F584" s="3" t="n">
-        <v>78.58</v>
+        <v>60.59</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
-      <c r="I584" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J584" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I584" s="2" t="inlineStr"/>
+      <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25859,75 +25849,71 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>62.95</v>
+        <v>6.13</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>-0.0008</v>
+        <v>0.0016</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>539710</v>
-      </c>
-      <c r="E585" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>8730000</v>
+      </c>
+      <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>56.09</v>
+        <v>61.01</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
       <c r="I585" s="6" t="inlineStr"/>
-      <c r="J585" s="8" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L585" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L585" s="6" t="inlineStr"/>
       <c r="M585" s="6" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>4.73</v>
+        <v>2.74</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.0216</v>
+        <v>-0.0108</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>62450000</v>
+        <v>98340000</v>
       </c>
       <c r="E586" s="4" t="n">
-        <v>0.8667</v>
+        <v>0.7119</v>
       </c>
       <c r="F586" s="3" t="n">
-        <v>77.90000000000001</v>
+        <v>43.27</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
-      <c r="I586" s="2" t="inlineStr"/>
-      <c r="J586" s="2" t="inlineStr"/>
+      <c r="I586" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J586" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25935,133 +25921,151 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>169</v>
+        <v>7.59</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0236</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>12070000</v>
-      </c>
-      <c r="E587" s="6" t="inlineStr"/>
+        <v>477650</v>
+      </c>
+      <c r="E587" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F587" s="7" t="n">
-        <v>60.59</v>
+        <v>39.58</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="6" t="inlineStr"/>
-      <c r="J587" s="6" t="inlineStr"/>
+      <c r="I587" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J587" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr"/>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>81.84</v>
+        <v>90.84999999999999</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0027</v>
+        <v>-0.0595</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>11800000</v>
+        <v>14880000</v>
       </c>
       <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>45.85</v>
+        <v>61.35</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
       <c r="J588" s="2" t="inlineStr"/>
-      <c r="K588" s="2" t="inlineStr"/>
-      <c r="L588" s="2" t="inlineStr"/>
+      <c r="K588" s="2" t="inlineStr">
+        <is>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>80.95</v>
+        <v>6.95</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0247</v>
+        <v>-0.09970000000000001</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>32400</v>
+        <v>75580000</v>
       </c>
       <c r="E589" s="8" t="n">
-        <v>0.58</v>
+        <v>0.1672</v>
       </c>
       <c r="F589" s="7" t="n">
-        <v>41.16</v>
+        <v>78.58</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
       <c r="I589" s="8" t="n">
-        <v>-9.409700000000001</v>
+        <v>-5.3262</v>
       </c>
       <c r="J589" s="8" t="n">
-        <v>-4.155</v>
+        <v>-4.2562</v>
       </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>2.82</v>
+        <v>62.95</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0537</v>
+        <v>-0.0008</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>263430000</v>
-      </c>
-      <c r="E590" s="2" t="inlineStr"/>
+        <v>539710</v>
+      </c>
+      <c r="E590" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F590" s="3" t="n">
-        <v>52.07</v>
+        <v>56.09</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="2" t="inlineStr"/>
-      <c r="J590" s="2" t="inlineStr"/>
+      <c r="J590" s="4" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26069,38 +26073,34 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>10.56</v>
+        <v>13.89</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.08529999999999999</v>
+        <v>0.0102</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>255670000</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.2479</v>
-      </c>
+        <v>35540000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>53.86</v>
+        <v>54.23</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="8" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
+      <c r="I591" s="6" t="inlineStr"/>
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26145,23 +26145,21 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>251</v>
+        <v>39.64</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0346</v>
+        <v>0.0195</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>8590</v>
-      </c>
-      <c r="E593" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>12770000</v>
+      </c>
+      <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>46.72</v>
+        <v>52.02</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26169,30 +26167,34 @@
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>197.4</v>
+        <v>24.62</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.099</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>20610000</v>
+        <v>15600000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>45.87</v>
+        <v>56.05</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26200,12 +26202,12 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26213,21 +26215,21 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>41.38</v>
+        <v>2.82</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0222</v>
+        <v>-0.0537</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>10990000</v>
+        <v>263430000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>60.95</v>
+        <v>52.07</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
@@ -26235,12 +26237,12 @@
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26248,34 +26250,40 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>33.9</v>
+        <v>152.1</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0174</v>
+        <v>-0.0225</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>4590000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>2330000</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>54.07</v>
+        <v>52.17</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J596" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26283,42 +26291,34 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>17.32</v>
+        <v>197.4</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0058</v>
+        <v>-0.099</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>12210000</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>20610000</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>47.99</v>
-      </c>
-      <c r="G597" s="7" t="n">
-        <v>163.71</v>
-      </c>
+        <v>45.87</v>
+      </c>
+      <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J597" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I597" s="6" t="inlineStr"/>
+      <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26326,21 +26326,21 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>90.84999999999999</v>
+        <v>33.9</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0595</v>
+        <v>-0.0174</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>14880000</v>
+        <v>4590000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>61.35</v>
+        <v>54.07</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26348,12 +26348,12 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26361,21 +26361,23 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>39.64</v>
+        <v>251</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0195</v>
+        <v>-0.0346</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>12770000</v>
-      </c>
-      <c r="E599" s="6" t="inlineStr"/>
+        <v>8590</v>
+      </c>
+      <c r="E599" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F599" s="7" t="n">
-        <v>52.02</v>
+        <v>46.72</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26383,47 +26385,51 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>24.62</v>
+        <v>17.32</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.004099999999999999</v>
+        <v>0.0058</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>15600000</v>
-      </c>
-      <c r="E600" s="2" t="inlineStr"/>
+        <v>12210000</v>
+      </c>
+      <c r="E600" s="4" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F600" s="3" t="n">
-        <v>56.05</v>
-      </c>
-      <c r="G600" s="2" t="inlineStr"/>
+        <v>47.99</v>
+      </c>
+      <c r="G600" s="3" t="n">
+        <v>163.71</v>
+      </c>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="2" t="inlineStr"/>
-      <c r="J600" s="2" t="inlineStr"/>
+      <c r="I600" s="4" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J600" s="4" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26431,108 +26437,92 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>13.89</v>
+        <v>103.5</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0102</v>
+        <v>-0.001</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>35540000</v>
+        <v>398550</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
-      <c r="F601" s="7" t="n">
-        <v>54.23</v>
-      </c>
+      <c r="F601" s="6" t="inlineStr"/>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>18.99</v>
+        <v>81.84</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0495</v>
+        <v>0.0027</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>102290000</v>
+        <v>11800000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
-      <c r="F602" s="2" t="inlineStr"/>
+      <c r="F602" s="3" t="n">
+        <v>45.85</v>
+      </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
       <c r="J602" s="2" t="inlineStr"/>
-      <c r="K602" s="2" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="K602" s="2" t="inlineStr"/>
+      <c r="L602" s="2" t="inlineStr"/>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>2.74</v>
+        <v>4.73</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0108</v>
+        <v>0.0216</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>98340000</v>
+        <v>62450000</v>
       </c>
       <c r="E603" s="8" t="n">
-        <v>0.7119</v>
+        <v>0.8667</v>
       </c>
       <c r="F603" s="7" t="n">
-        <v>43.27</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26540,20 +26530,22 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>103.5</v>
+        <v>16.08</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.001</v>
+        <v>-0.0111</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>398550</v>
+        <v>72700000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
-      <c r="F604" s="2" t="inlineStr"/>
+      <c r="F604" s="3" t="n">
+        <v>51.02</v>
+      </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="2" t="inlineStr"/>
@@ -26563,40 +26555,48 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L604" s="2" t="inlineStr"/>
+      <c r="L604" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>16.08</v>
+        <v>10.56</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0111</v>
+        <v>0.08529999999999999</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>72700000</v>
-      </c>
-      <c r="E605" s="6" t="inlineStr"/>
+        <v>255670000</v>
+      </c>
+      <c r="E605" s="8" t="n">
+        <v>0.2479</v>
+      </c>
       <c r="F605" s="7" t="n">
-        <v>51.02</v>
+        <v>53.86</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="6" t="inlineStr"/>
+      <c r="I605" s="8" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26604,21 +26604,21 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>6.13</v>
+        <v>41.38</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0016</v>
+        <v>0.0222</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>8730000</v>
+        <v>10990000</v>
       </c>
       <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>61.01</v>
+        <v>60.95</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26626,51 +26626,51 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>152.1</v>
+        <v>80.95</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0225</v>
+        <v>0.0247</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>2330000</v>
+        <v>32400</v>
       </c>
       <c r="E607" s="8" t="n">
-        <v>0.1071</v>
+        <v>0.58</v>
       </c>
       <c r="F607" s="7" t="n">
-        <v>52.17</v>
+        <v>41.16</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
       <c r="I607" s="8" t="n">
-        <v>-3.6635</v>
+        <v>-9.409700000000001</v>
       </c>
       <c r="J607" s="8" t="n">
-        <v>-0.4897</v>
+        <v>-4.155</v>
       </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr"/>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26695,7 +26695,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>23.04.2026 10:30</t>
+          <t>23.04.2026 11:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 23.04.2026 12:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-23.xlsx
+++ b/data/bist_screener_2026-04-23.xlsx
@@ -25781,32 +25781,40 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>18.99</v>
+        <v>2.74</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>-0.0495</v>
+        <v>-0.0108</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>102290000</v>
-      </c>
-      <c r="E583" s="6" t="inlineStr"/>
-      <c r="F583" s="6" t="inlineStr"/>
+        <v>98340000</v>
+      </c>
+      <c r="E583" s="8" t="n">
+        <v>0.7119</v>
+      </c>
+      <c r="F583" s="7" t="n">
+        <v>43.27</v>
+      </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
-      <c r="I583" s="6" t="inlineStr"/>
-      <c r="J583" s="6" t="inlineStr"/>
+      <c r="I583" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J583" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L583" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M583" s="6" t="inlineStr"/>
@@ -25814,21 +25822,21 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>169</v>
+        <v>197.4</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>0.0236</v>
+        <v>-0.099</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>12070000</v>
+        <v>20610000</v>
       </c>
       <c r="E584" s="2" t="inlineStr"/>
       <c r="F584" s="3" t="n">
-        <v>60.59</v>
+        <v>45.87</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
@@ -25836,12 +25844,12 @@
       <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25849,21 +25857,21 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>6.13</v>
+        <v>16.08</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.0016</v>
+        <v>-0.0111</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>8730000</v>
+        <v>72700000</v>
       </c>
       <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>61.01</v>
+        <v>51.02</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
@@ -25874,105 +25882,111 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L585" s="6" t="inlineStr"/>
+      <c r="L585" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M585" s="6" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>2.74</v>
+        <v>7.59</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.0108</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>98340000</v>
+        <v>477650</v>
       </c>
       <c r="E586" s="4" t="n">
-        <v>0.7119</v>
+        <v>0.95</v>
       </c>
       <c r="F586" s="3" t="n">
-        <v>43.27</v>
+        <v>39.58</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
       <c r="I586" s="4" t="n">
-        <v>-191.6342</v>
+        <v>-23.6291</v>
       </c>
       <c r="J586" s="4" t="n">
-        <v>-0.8093</v>
+        <v>-0.4678</v>
       </c>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L586" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L586" s="2" t="inlineStr"/>
       <c r="M586" s="2" t="inlineStr"/>
     </row>
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>7.59</v>
+        <v>152.1</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.007800000000000001</v>
+        <v>-0.0225</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>477650</v>
+        <v>2330000</v>
       </c>
       <c r="E587" s="8" t="n">
-        <v>0.95</v>
+        <v>0.1071</v>
       </c>
       <c r="F587" s="7" t="n">
-        <v>39.58</v>
+        <v>52.17</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
       <c r="I587" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-3.6635</v>
       </c>
       <c r="J587" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-0.4897</v>
       </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>90.84999999999999</v>
+        <v>251</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0595</v>
+        <v>-0.0346</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>14880000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>8590</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>61.35</v>
+        <v>46.72</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25980,53 +25994,43 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr"/>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>6.95</v>
+        <v>13.89</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.09970000000000001</v>
+        <v>0.0102</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>75580000</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>35540000</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>78.58</v>
+        <v>54.23</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J589" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I589" s="6" t="inlineStr"/>
+      <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26034,38 +26038,40 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>62.95</v>
+        <v>6.95</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0008</v>
+        <v>-0.09970000000000001</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>539710</v>
+        <v>75580000</v>
       </c>
       <c r="E590" s="4" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.1672</v>
       </c>
       <c r="F590" s="3" t="n">
-        <v>56.09</v>
+        <v>78.58</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="2" t="inlineStr"/>
+      <c r="I590" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
       <c r="J590" s="4" t="n">
-        <v>0.4139</v>
+        <v>-4.2562</v>
       </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26073,21 +26079,23 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>13.89</v>
+        <v>28.66</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0102</v>
+        <v>-0.0478</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>35540000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>18930000</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>54.23</v>
+        <v>50.42</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26095,12 +26103,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26108,36 +26116,42 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>28.66</v>
+        <v>17.32</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0478</v>
+        <v>0.0058</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>18930000</v>
+        <v>12210000</v>
       </c>
       <c r="E592" s="4" t="n">
-        <v>0.2667</v>
+        <v>0.9246</v>
       </c>
       <c r="F592" s="3" t="n">
-        <v>50.42</v>
-      </c>
-      <c r="G592" s="2" t="inlineStr"/>
+        <v>47.99</v>
+      </c>
+      <c r="G592" s="3" t="n">
+        <v>163.71</v>
+      </c>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="2" t="inlineStr"/>
+      <c r="I592" s="4" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J592" s="4" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26145,21 +26159,21 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>39.64</v>
+        <v>33.9</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0195</v>
+        <v>-0.0174</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>12770000</v>
+        <v>4590000</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>52.02</v>
+        <v>54.07</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26167,12 +26181,12 @@
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26180,34 +26194,38 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>24.62</v>
+        <v>62.95</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.004099999999999999</v>
+        <v>-0.0008</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>15600000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>539710</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>56.05</v>
+        <v>56.09</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
       <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="J594" s="4" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26215,22 +26233,20 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>2.82</v>
+        <v>18.99</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0537</v>
+        <v>-0.0495</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>263430000</v>
+        <v>102290000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
-      <c r="F595" s="7" t="n">
-        <v>52.07</v>
-      </c>
+      <c r="F595" s="6" t="inlineStr"/>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
@@ -26242,7 +26258,7 @@
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26250,62 +26266,48 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>152.1</v>
+        <v>81.84</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0225</v>
+        <v>0.0027</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>2330000</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>11800000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>52.17</v>
+        <v>45.85</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J596" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
-      <c r="K596" s="2" t="inlineStr">
-        <is>
-          <t>Perakende satış</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
-        </is>
-      </c>
+      <c r="I596" s="2" t="inlineStr"/>
+      <c r="J596" s="2" t="inlineStr"/>
+      <c r="K596" s="2" t="inlineStr"/>
+      <c r="L596" s="2" t="inlineStr"/>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>197.4</v>
+        <v>41.38</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.099</v>
+        <v>0.0222</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>20610000</v>
+        <v>10990000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>45.87</v>
+        <v>60.95</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26313,12 +26315,12 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26326,21 +26328,21 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>33.9</v>
+        <v>2.82</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0174</v>
+        <v>-0.0537</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>4590000</v>
+        <v>263430000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>54.07</v>
+        <v>52.07</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26348,12 +26350,12 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26361,23 +26363,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>251</v>
+        <v>39.64</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0346</v>
+        <v>0.0195</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>8590</v>
-      </c>
-      <c r="E599" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>12770000</v>
+      </c>
+      <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>46.72</v>
+        <v>52.02</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26385,51 +26385,47 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+        </is>
+      </c>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>17.32</v>
+        <v>24.62</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0058</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>12210000</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>15600000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>47.99</v>
-      </c>
-      <c r="G600" s="3" t="n">
-        <v>163.71</v>
-      </c>
+        <v>56.05</v>
+      </c>
+      <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26437,79 +26433,93 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>103.5</v>
+        <v>90.84999999999999</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.001</v>
+        <v>-0.0595</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>398550</v>
+        <v>14880000</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
-      <c r="F601" s="6" t="inlineStr"/>
+      <c r="F601" s="7" t="n">
+        <v>61.35</v>
+      </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>81.84</v>
+        <v>4.73</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0027</v>
+        <v>0.0216</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>11800000</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>62450000</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>45.85</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
       <c r="J602" s="2" t="inlineStr"/>
-      <c r="K602" s="2" t="inlineStr"/>
-      <c r="L602" s="2" t="inlineStr"/>
+      <c r="K602" s="2" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>4.73</v>
+        <v>6.13</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0216</v>
+        <v>0.0016</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>62450000</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>8730000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>77.90000000000001</v>
+        <v>61.01</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26520,44 +26530,44 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
-        </is>
-      </c>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>16.08</v>
+        <v>10.56</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0111</v>
+        <v>0.08529999999999999</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>72700000</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>255670000</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>0.2479</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>51.02</v>
+        <v>53.86</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="2" t="inlineStr"/>
+      <c r="I604" s="4" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26565,60 +26575,58 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>10.56</v>
+        <v>80.95</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.08529999999999999</v>
+        <v>0.0247</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>255670000</v>
+        <v>32400</v>
       </c>
       <c r="E605" s="8" t="n">
-        <v>0.2479</v>
+        <v>0.58</v>
       </c>
       <c r="F605" s="7" t="n">
-        <v>53.86</v>
+        <v>41.16</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="8" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
-      <c r="J605" s="6" t="inlineStr"/>
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J605" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>41.38</v>
+        <v>169</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0222</v>
+        <v>0.0236</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>10990000</v>
+        <v>12070000</v>
       </c>
       <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>60.95</v>
+        <v>60.59</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26626,12 +26634,12 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26639,35 +26647,27 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>80.95</v>
+        <v>103.5</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0247</v>
+        <v>-0.001</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>32400</v>
-      </c>
-      <c r="E607" s="8" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="F607" s="7" t="n">
-        <v>41.16</v>
-      </c>
+        <v>398550</v>
+      </c>
+      <c r="E607" s="6" t="inlineStr"/>
+      <c r="F607" s="6" t="inlineStr"/>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J607" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I607" s="6" t="inlineStr"/>
+      <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr"/>
@@ -26695,7 +26695,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>23.04.2026 11:30</t>
+          <t>23.04.2026 12:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 23.04.2026 13:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-23.xlsx
+++ b/data/bist_screener_2026-04-23.xlsx
@@ -25781,40 +25781,34 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>2.74</v>
+        <v>39.64</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>-0.0108</v>
+        <v>0.0195</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>98340000</v>
-      </c>
-      <c r="E583" s="8" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>12770000</v>
+      </c>
+      <c r="E583" s="6" t="inlineStr"/>
       <c r="F583" s="7" t="n">
-        <v>43.27</v>
+        <v>52.02</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
-      <c r="I583" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J583" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I583" s="6" t="inlineStr"/>
+      <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L583" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M583" s="6" t="inlineStr"/>
@@ -25822,21 +25816,21 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>197.4</v>
+        <v>33.9</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.099</v>
+        <v>-0.0174</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>20610000</v>
+        <v>4590000</v>
       </c>
       <c r="E584" s="2" t="inlineStr"/>
       <c r="F584" s="3" t="n">
-        <v>45.87</v>
+        <v>54.07</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
@@ -25844,12 +25838,12 @@
       <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25857,21 +25851,21 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>16.08</v>
+        <v>197.4</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>-0.0111</v>
+        <v>-0.099</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>72700000</v>
+        <v>20610000</v>
       </c>
       <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>51.02</v>
+        <v>45.87</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
@@ -25879,12 +25873,12 @@
       <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25892,77 +25886,77 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>7.59</v>
+        <v>17.32</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.007800000000000001</v>
+        <v>0.0058</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>477650</v>
+        <v>12210000</v>
       </c>
       <c r="E586" s="4" t="n">
-        <v>0.95</v>
+        <v>0.9246</v>
       </c>
       <c r="F586" s="3" t="n">
-        <v>39.58</v>
-      </c>
-      <c r="G586" s="2" t="inlineStr"/>
+        <v>47.99</v>
+      </c>
+      <c r="G586" s="3" t="n">
+        <v>163.71</v>
+      </c>
       <c r="H586" s="2" t="inlineStr"/>
       <c r="I586" s="4" t="n">
-        <v>-23.6291</v>
+        <v>0.0028</v>
       </c>
       <c r="J586" s="4" t="n">
-        <v>-0.4678</v>
+        <v>-10.3171</v>
       </c>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L586" s="2" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L586" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+        </is>
+      </c>
       <c r="M586" s="2" t="inlineStr"/>
     </row>
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>152.1</v>
+        <v>13.89</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.0225</v>
+        <v>0.0102</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>2330000</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>35540000</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>52.17</v>
+        <v>54.23</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J587" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I587" s="6" t="inlineStr"/>
+      <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25970,23 +25964,21 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>251</v>
+        <v>6.13</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0346</v>
+        <v>0.0016</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>8590</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>8730000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>46.72</v>
+        <v>61.01</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25994,7 +25986,7 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr"/>
@@ -26003,34 +25995,38 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>13.89</v>
+        <v>62.95</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0102</v>
+        <v>-0.0008</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>35540000</v>
-      </c>
-      <c r="E589" s="6" t="inlineStr"/>
+        <v>539710</v>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F589" s="7" t="n">
-        <v>54.23</v>
+        <v>56.09</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
       <c r="I589" s="6" t="inlineStr"/>
-      <c r="J589" s="6" t="inlineStr"/>
+      <c r="J589" s="8" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26038,64 +26034,48 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>6.95</v>
+        <v>81.84</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.09970000000000001</v>
+        <v>0.0027</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>75580000</v>
-      </c>
-      <c r="E590" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>11800000</v>
+      </c>
+      <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>78.58</v>
+        <v>45.85</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J590" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
-      <c r="K590" s="2" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="I590" s="2" t="inlineStr"/>
+      <c r="J590" s="2" t="inlineStr"/>
+      <c r="K590" s="2" t="inlineStr"/>
+      <c r="L590" s="2" t="inlineStr"/>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>28.66</v>
+        <v>16.08</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0478</v>
+        <v>-0.0111</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>18930000</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>72700000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>50.42</v>
+        <v>51.02</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26103,12 +26083,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26116,77 +26096,65 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>17.32</v>
+        <v>251</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0058</v>
+        <v>-0.0346</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>12210000</v>
+        <v>8590</v>
       </c>
       <c r="E592" s="4" t="n">
-        <v>0.9246</v>
+        <v>0.2578</v>
       </c>
       <c r="F592" s="3" t="n">
-        <v>47.99</v>
-      </c>
-      <c r="G592" s="3" t="n">
-        <v>163.71</v>
-      </c>
+        <v>46.72</v>
+      </c>
+      <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J592" s="4" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I592" s="2" t="inlineStr"/>
+      <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr"/>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>33.9</v>
+        <v>18.99</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0174</v>
+        <v>-0.0495</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>4590000</v>
+        <v>102290000</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
-      <c r="F593" s="7" t="n">
-        <v>54.07</v>
-      </c>
+      <c r="F593" s="6" t="inlineStr"/>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="6" t="inlineStr"/>
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26194,38 +26162,34 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>62.95</v>
+        <v>2.82</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0008</v>
+        <v>-0.0537</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>539710</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>263430000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>56.09</v>
+        <v>52.07</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
       <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="4" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26233,17 +26197,17 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>18.99</v>
+        <v>103.5</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0495</v>
+        <v>-0.001</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>102290000</v>
+        <v>398550</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="6" t="inlineStr"/>
@@ -26256,38 +26220,44 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L595" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="L595" s="6" t="inlineStr"/>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>81.84</v>
+        <v>28.66</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0027</v>
+        <v>-0.0478</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>11800000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>18930000</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>45.85</v>
+        <v>50.42</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
       <c r="I596" s="2" t="inlineStr"/>
       <c r="J596" s="2" t="inlineStr"/>
-      <c r="K596" s="2" t="inlineStr"/>
-      <c r="L596" s="2" t="inlineStr"/>
+      <c r="K596" s="2" t="inlineStr">
+        <is>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
@@ -26328,34 +26298,40 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>2.82</v>
+        <v>2.74</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0537</v>
+        <v>-0.0108</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>263430000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>98340000</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>52.07</v>
+        <v>43.27</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="I598" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J598" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26363,34 +26339,38 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>39.64</v>
+        <v>10.56</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0195</v>
+        <v>0.08529999999999999</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>12770000</v>
-      </c>
-      <c r="E599" s="6" t="inlineStr"/>
+        <v>255670000</v>
+      </c>
+      <c r="E599" s="8" t="n">
+        <v>0.2479</v>
+      </c>
       <c r="F599" s="7" t="n">
-        <v>52.02</v>
+        <v>53.86</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="6" t="inlineStr"/>
+      <c r="I599" s="8" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26398,36 +26378,38 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>24.62</v>
+        <v>80.95</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.004099999999999999</v>
+        <v>0.0247</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>15600000</v>
-      </c>
-      <c r="E600" s="2" t="inlineStr"/>
+        <v>32400</v>
+      </c>
+      <c r="E600" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F600" s="3" t="n">
-        <v>56.05</v>
+        <v>41.16</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="2" t="inlineStr"/>
-      <c r="J600" s="2" t="inlineStr"/>
+      <c r="I600" s="4" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J600" s="4" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L600" s="2" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L600" s="2" t="inlineStr"/>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
@@ -26468,23 +26450,21 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>4.73</v>
+        <v>24.62</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0216</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>62450000</v>
-      </c>
-      <c r="E602" s="4" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>15600000</v>
+      </c>
+      <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>77.90000000000001</v>
+        <v>56.05</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26492,12 +26472,12 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26505,69 +26485,75 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>6.13</v>
+        <v>6.95</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0016</v>
+        <v>-0.09970000000000001</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>8730000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>75580000</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>61.01</v>
+        <v>78.58</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J603" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
         </is>
       </c>
-      <c r="L603" s="6" t="inlineStr"/>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>10.56</v>
+        <v>169</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.08529999999999999</v>
+        <v>0.0236</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>255670000</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.2479</v>
-      </c>
+        <v>12070000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>53.86</v>
+        <v>60.59</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="4" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
+      <c r="I604" s="2" t="inlineStr"/>
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26575,35 +26561,35 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>80.95</v>
+        <v>7.59</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0247</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>32400</v>
+        <v>477650</v>
       </c>
       <c r="E605" s="8" t="n">
-        <v>0.58</v>
+        <v>0.95</v>
       </c>
       <c r="F605" s="7" t="n">
-        <v>41.16</v>
+        <v>39.58</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="8" t="n">
-        <v>-9.409700000000001</v>
+        <v>-23.6291</v>
       </c>
       <c r="J605" s="8" t="n">
-        <v>-4.155</v>
+        <v>-0.4678</v>
       </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr"/>
@@ -26612,34 +26598,40 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>169</v>
+        <v>152.1</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0236</v>
+        <v>-0.0225</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>12070000</v>
-      </c>
-      <c r="E606" s="2" t="inlineStr"/>
+        <v>2330000</v>
+      </c>
+      <c r="E606" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F606" s="3" t="n">
-        <v>60.59</v>
+        <v>52.17</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="2" t="inlineStr"/>
+      <c r="I606" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J606" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26647,20 +26639,24 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>103.5</v>
+        <v>4.73</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.001</v>
+        <v>0.0216</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>398550</v>
-      </c>
-      <c r="E607" s="6" t="inlineStr"/>
-      <c r="F607" s="6" t="inlineStr"/>
+        <v>62450000</v>
+      </c>
+      <c r="E607" s="8" t="n">
+        <v>0.8667</v>
+      </c>
+      <c r="F607" s="7" t="n">
+        <v>77.90000000000001</v>
+      </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
       <c r="I607" s="6" t="inlineStr"/>
@@ -26670,7 +26666,11 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L607" s="6" t="inlineStr"/>
+      <c r="L607" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26695,7 +26695,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>23.04.2026 12:30</t>
+          <t>23.04.2026 13:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 23.04.2026 14:38 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-23.xlsx
+++ b/data/bist_screener_2026-04-23.xlsx
@@ -25781,21 +25781,21 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>39.64</v>
+        <v>6.13</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0.0195</v>
+        <v>0.0016</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>12770000</v>
+        <v>8730000</v>
       </c>
       <c r="E583" s="6" t="inlineStr"/>
       <c r="F583" s="7" t="n">
-        <v>52.02</v>
+        <v>61.01</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
@@ -25803,34 +25803,30 @@
       <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L583" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr"/>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>33.9</v>
+        <v>2.82</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0174</v>
+        <v>-0.0537</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>4590000</v>
+        <v>263430000</v>
       </c>
       <c r="E584" s="2" t="inlineStr"/>
       <c r="F584" s="3" t="n">
-        <v>54.07</v>
+        <v>52.07</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
@@ -25838,12 +25834,12 @@
       <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25851,34 +25847,38 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>197.4</v>
+        <v>10.56</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>-0.099</v>
+        <v>0.08529999999999999</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>20610000</v>
-      </c>
-      <c r="E585" s="6" t="inlineStr"/>
+        <v>255670000</v>
+      </c>
+      <c r="E585" s="8" t="n">
+        <v>0.2479</v>
+      </c>
       <c r="F585" s="7" t="n">
-        <v>45.87</v>
+        <v>53.86</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
-      <c r="I585" s="6" t="inlineStr"/>
+      <c r="I585" s="8" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
       <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25886,64 +25886,54 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>17.32</v>
+        <v>251</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.0058</v>
+        <v>-0.0346</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>12210000</v>
+        <v>8590</v>
       </c>
       <c r="E586" s="4" t="n">
-        <v>0.9246</v>
+        <v>0.2578</v>
       </c>
       <c r="F586" s="3" t="n">
-        <v>47.99</v>
-      </c>
-      <c r="G586" s="3" t="n">
-        <v>163.71</v>
-      </c>
+        <v>46.72</v>
+      </c>
+      <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
-      <c r="I586" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J586" s="4" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I586" s="2" t="inlineStr"/>
+      <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L586" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L586" s="2" t="inlineStr"/>
       <c r="M586" s="2" t="inlineStr"/>
     </row>
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>13.89</v>
+        <v>41.38</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0102</v>
+        <v>0.0222</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>35540000</v>
+        <v>10990000</v>
       </c>
       <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>54.23</v>
+        <v>60.95</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25951,12 +25941,12 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25964,29 +25954,35 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>6.13</v>
+        <v>80.95</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0016</v>
+        <v>0.0247</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>8730000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>32400</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>61.01</v>
+        <v>41.16</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J588" s="4" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Taşımacılık</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr"/>
@@ -25995,38 +25991,36 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>62.95</v>
+        <v>4.73</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0008</v>
+        <v>0.0216</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>539710</v>
+        <v>62450000</v>
       </c>
       <c r="E589" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.8667</v>
       </c>
       <c r="F589" s="7" t="n">
-        <v>56.09</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
       <c r="I589" s="6" t="inlineStr"/>
-      <c r="J589" s="8" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26034,61 +26028,75 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>81.84</v>
+        <v>90.84999999999999</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0027</v>
+        <v>-0.0595</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>11800000</v>
+        <v>14880000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>45.85</v>
+        <v>61.35</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="2" t="inlineStr"/>
       <c r="J590" s="2" t="inlineStr"/>
-      <c r="K590" s="2" t="inlineStr"/>
-      <c r="L590" s="2" t="inlineStr"/>
+      <c r="K590" s="2" t="inlineStr">
+        <is>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>16.08</v>
+        <v>152.1</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0111</v>
+        <v>-0.0225</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>72700000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>2330000</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>51.02</v>
+        <v>52.17</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="I591" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J591" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26096,23 +26104,21 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>251</v>
+        <v>16.08</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0346</v>
+        <v>-0.0111</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>8590</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>72700000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>46.72</v>
+        <v>51.02</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26120,41 +26126,47 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>18.99</v>
+        <v>197.4</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0495</v>
+        <v>-0.099</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>102290000</v>
+        <v>20610000</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
-      <c r="F593" s="6" t="inlineStr"/>
+      <c r="F593" s="7" t="n">
+        <v>45.87</v>
+      </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="6" t="inlineStr"/>
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26162,26 +26174,32 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>2.82</v>
+        <v>6.95</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0537</v>
+        <v>-0.09970000000000001</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>263430000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>75580000</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>52.07</v>
+        <v>78.58</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26189,7 +26207,7 @@
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26197,141 +26215,141 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>103.5</v>
+        <v>28.66</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.001</v>
+        <v>-0.0478</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>398550</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
-      <c r="F595" s="6" t="inlineStr"/>
+        <v>18930000</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.2667</v>
+      </c>
+      <c r="F595" s="7" t="n">
+        <v>50.42</v>
+      </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>28.66</v>
+        <v>7.59</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0478</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>18930000</v>
+        <v>477650</v>
       </c>
       <c r="E596" s="4" t="n">
-        <v>0.2667</v>
+        <v>0.95</v>
       </c>
       <c r="F596" s="3" t="n">
-        <v>50.42</v>
+        <v>39.58</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J596" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr"/>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>41.38</v>
+        <v>103.5</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0222</v>
+        <v>-0.001</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>10990000</v>
+        <v>398550</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
-      <c r="F597" s="7" t="n">
-        <v>60.95</v>
-      </c>
+      <c r="F597" s="6" t="inlineStr"/>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
       <c r="I597" s="6" t="inlineStr"/>
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>2.74</v>
+        <v>62.95</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0108</v>
+        <v>-0.0008</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>98340000</v>
+        <v>539710</v>
       </c>
       <c r="E598" s="4" t="n">
-        <v>0.7119</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F598" s="3" t="n">
-        <v>43.27</v>
+        <v>56.09</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
+      <c r="I598" s="2" t="inlineStr"/>
       <c r="J598" s="4" t="n">
-        <v>-0.8093</v>
+        <v>0.4139</v>
       </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26339,38 +26357,40 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>10.56</v>
+        <v>2.74</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.08529999999999999</v>
+        <v>-0.0108</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>255670000</v>
+        <v>98340000</v>
       </c>
       <c r="E599" s="8" t="n">
-        <v>0.2479</v>
+        <v>0.7119</v>
       </c>
       <c r="F599" s="7" t="n">
-        <v>53.86</v>
+        <v>43.27</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="8" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
-      <c r="J599" s="6" t="inlineStr"/>
+        <v>-191.6342</v>
+      </c>
+      <c r="J599" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26378,58 +26398,56 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>80.95</v>
+        <v>169</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0247</v>
+        <v>0.0236</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>32400</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>12070000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>41.16</v>
+        <v>60.59</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L600" s="2" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L600" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+        </is>
+      </c>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>90.84999999999999</v>
+        <v>33.9</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0595</v>
+        <v>-0.0174</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>14880000</v>
+        <v>4590000</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>61.35</v>
+        <v>54.07</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
@@ -26437,12 +26455,12 @@
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26450,34 +26468,32 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>24.62</v>
+        <v>18.99</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.004099999999999999</v>
+        <v>-0.0495</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>15600000</v>
+        <v>102290000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
-      <c r="F602" s="3" t="n">
-        <v>56.05</v>
-      </c>
+      <c r="F602" s="2" t="inlineStr"/>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26485,40 +26501,34 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>6.95</v>
+        <v>39.64</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.09970000000000001</v>
+        <v>0.0195</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>75580000</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>12770000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>78.58</v>
+        <v>52.02</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26526,112 +26536,96 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>169</v>
+        <v>81.84</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0236</v>
+        <v>0.0027</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>12070000</v>
+        <v>11800000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>60.59</v>
+        <v>45.85</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="2" t="inlineStr"/>
       <c r="J604" s="2" t="inlineStr"/>
-      <c r="K604" s="2" t="inlineStr">
-        <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+      <c r="K604" s="2" t="inlineStr"/>
+      <c r="L604" s="2" t="inlineStr"/>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>7.59</v>
+        <v>24.62</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.007800000000000001</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>477650</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>15600000</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>39.58</v>
+        <v>56.05</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J605" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I605" s="6" t="inlineStr"/>
+      <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr"/>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>152.1</v>
+        <v>13.89</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0225</v>
+        <v>0.0102</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>2330000</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>35540000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>52.17</v>
+        <v>54.23</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J606" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26639,36 +26633,42 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>4.73</v>
+        <v>17.32</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0216</v>
+        <v>0.0058</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>62450000</v>
+        <v>12210000</v>
       </c>
       <c r="E607" s="8" t="n">
-        <v>0.8667</v>
+        <v>0.9246</v>
       </c>
       <c r="F607" s="7" t="n">
-        <v>77.90000000000001</v>
-      </c>
-      <c r="G607" s="6" t="inlineStr"/>
+        <v>47.99</v>
+      </c>
+      <c r="G607" s="7" t="n">
+        <v>163.71</v>
+      </c>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="6" t="inlineStr"/>
-      <c r="J607" s="6" t="inlineStr"/>
+      <c r="I607" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J607" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26695,7 +26695,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>23.04.2026 13:30</t>
+          <t>23.04.2026 14:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 23.04.2026 16:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-23.xlsx
+++ b/data/bist_screener_2026-04-23.xlsx
@@ -25824,21 +25824,23 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>197.4</v>
+        <v>28.66</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.099</v>
+        <v>-0.0478</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>20610000</v>
-      </c>
-      <c r="E584" s="2" t="inlineStr"/>
+        <v>18930000</v>
+      </c>
+      <c r="E584" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F584" s="3" t="n">
-        <v>45.87</v>
+        <v>50.42</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
@@ -25851,7 +25853,7 @@
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25859,21 +25861,21 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>24.62</v>
+        <v>13.89</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.004099999999999999</v>
+        <v>0.0102</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>15600000</v>
+        <v>35540000</v>
       </c>
       <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>56.05</v>
+        <v>54.23</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
@@ -25881,12 +25883,12 @@
       <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25894,21 +25896,21 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>90.84999999999999</v>
+        <v>41.38</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.0595</v>
+        <v>0.0222</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>14880000</v>
+        <v>10990000</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>61.35</v>
+        <v>60.95</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25916,12 +25918,12 @@
       <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25929,21 +25931,21 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>39.64</v>
+        <v>169</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0195</v>
+        <v>0.0236</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>12770000</v>
+        <v>12070000</v>
       </c>
       <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>52.02</v>
+        <v>60.59</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25951,7 +25953,7 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
@@ -25964,42 +25966,32 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>17.32</v>
+        <v>18.99</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0058</v>
+        <v>-0.0495</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>12210000</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.9246</v>
-      </c>
-      <c r="F588" s="3" t="n">
-        <v>47.99</v>
-      </c>
-      <c r="G588" s="3" t="n">
-        <v>163.71</v>
-      </c>
+        <v>102290000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
+      <c r="F588" s="2" t="inlineStr"/>
+      <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J588" s="4" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I588" s="2" t="inlineStr"/>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -26007,34 +25999,40 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>33.9</v>
+        <v>6.95</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0174</v>
+        <v>-0.09970000000000001</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>4590000</v>
-      </c>
-      <c r="E589" s="6" t="inlineStr"/>
+        <v>75580000</v>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F589" s="7" t="n">
-        <v>54.07</v>
+        <v>78.58</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="6" t="inlineStr"/>
-      <c r="J589" s="6" t="inlineStr"/>
+      <c r="I589" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J589" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26042,157 +26040,161 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>80.95</v>
+        <v>4.73</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0247</v>
+        <v>0.0216</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>32400</v>
+        <v>62450000</v>
       </c>
       <c r="E590" s="4" t="n">
-        <v>0.58</v>
+        <v>0.8667</v>
       </c>
       <c r="F590" s="3" t="n">
-        <v>41.16</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J590" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I590" s="2" t="inlineStr"/>
+      <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>41.38</v>
+        <v>7.59</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0222</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>10990000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>477650</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>60.95</v>
+        <v>39.58</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="I591" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J591" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr"/>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>4.73</v>
+        <v>81.84</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0216</v>
+        <v>0.0027</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>62450000</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>11800000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>77.90000000000001</v>
+        <v>45.85</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="2" t="inlineStr"/>
       <c r="J592" s="2" t="inlineStr"/>
-      <c r="K592" s="2" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
-        </is>
-      </c>
+      <c r="K592" s="2" t="inlineStr"/>
+      <c r="L592" s="2" t="inlineStr"/>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>81.84</v>
+        <v>62.95</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0027</v>
+        <v>-0.0008</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>11800000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>539710</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>45.85</v>
+        <v>56.09</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
-      <c r="K593" s="6" t="inlineStr"/>
-      <c r="L593" s="6" t="inlineStr"/>
+      <c r="J593" s="8" t="n">
+        <v>0.4139</v>
+      </c>
+      <c r="K593" s="6" t="inlineStr">
+        <is>
+          <t>Teknoloji hizmetleri</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>2.82</v>
+        <v>197.4</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0537</v>
+        <v>-0.099</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>263430000</v>
+        <v>20610000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>52.07</v>
+        <v>45.87</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26200,12 +26202,12 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26213,67 +26215,83 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>103.5</v>
+        <v>17.32</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.001</v>
+        <v>0.0058</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>398550</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
-      <c r="F595" s="6" t="inlineStr"/>
-      <c r="G595" s="6" t="inlineStr"/>
+        <v>12210000</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.9246</v>
+      </c>
+      <c r="F595" s="7" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="G595" s="7" t="n">
+        <v>163.71</v>
+      </c>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="I595" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J595" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+        </is>
+      </c>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>62.95</v>
+        <v>2.74</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0008</v>
+        <v>-0.0108</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>539710</v>
+        <v>98340000</v>
       </c>
       <c r="E596" s="4" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.7119</v>
       </c>
       <c r="F596" s="3" t="n">
-        <v>56.09</v>
+        <v>43.27</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
       <c r="J596" s="4" t="n">
-        <v>0.4139</v>
+        <v>-0.8093</v>
       </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26281,58 +26299,58 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>13.89</v>
+        <v>80.95</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0102</v>
+        <v>0.0247</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>35540000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>32400</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>54.23</v>
+        <v>41.16</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>251</v>
+        <v>2.82</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0346</v>
+        <v>-0.0537</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>8590</v>
-      </c>
-      <c r="E598" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>263430000</v>
+      </c>
+      <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>46.72</v>
+        <v>52.07</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26340,30 +26358,34 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>6.13</v>
+        <v>16.08</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0016</v>
+        <v>-0.0111</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>8730000</v>
+        <v>72700000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>61.01</v>
+        <v>51.02</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26374,112 +26396,114 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L599" s="6" t="inlineStr"/>
+      <c r="L599" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>7.59</v>
+        <v>152.1</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.007800000000000001</v>
+        <v>-0.0225</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>477650</v>
+        <v>2330000</v>
       </c>
       <c r="E600" s="4" t="n">
-        <v>0.95</v>
+        <v>0.1071</v>
       </c>
       <c r="F600" s="3" t="n">
-        <v>39.58</v>
+        <v>52.17</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="4" t="n">
-        <v>-23.6291</v>
+        <v>-3.6635</v>
       </c>
       <c r="J600" s="4" t="n">
-        <v>-0.4678</v>
+        <v>-0.4897</v>
       </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L600" s="2" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L600" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>28.66</v>
+        <v>103.5</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0478</v>
+        <v>-0.001</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>18930000</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.2667</v>
-      </c>
-      <c r="F601" s="7" t="n">
-        <v>50.42</v>
-      </c>
+        <v>398550</v>
+      </c>
+      <c r="E601" s="6" t="inlineStr"/>
+      <c r="F601" s="6" t="inlineStr"/>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>18.99</v>
+        <v>33.9</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0495</v>
+        <v>-0.0174</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>102290000</v>
+        <v>4590000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
-      <c r="F602" s="2" t="inlineStr"/>
+      <c r="F602" s="3" t="n">
+        <v>54.07</v>
+      </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26487,40 +26511,34 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>2.74</v>
+        <v>39.64</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0108</v>
+        <v>0.0195</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>98340000</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>12770000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>43.27</v>
+        <v>52.02</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26528,40 +26546,34 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>6.95</v>
+        <v>90.84999999999999</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.09970000000000001</v>
+        <v>-0.0595</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>75580000</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>14880000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>78.58</v>
+        <v>61.35</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J604" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I604" s="2" t="inlineStr"/>
+      <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26569,21 +26581,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>16.08</v>
+        <v>24.62</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0111</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>72700000</v>
+        <v>15600000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>51.02</v>
+        <v>56.05</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26591,12 +26603,12 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26604,21 +26616,23 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>169</v>
+        <v>251</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0236</v>
+        <v>-0.0346</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>12070000</v>
-      </c>
-      <c r="E606" s="2" t="inlineStr"/>
+        <v>8590</v>
+      </c>
+      <c r="E606" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F606" s="3" t="n">
-        <v>60.59</v>
+        <v>46.72</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26626,55 +26640,41 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>152.1</v>
+        <v>6.13</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0225</v>
+        <v>0.0016</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>2330000</v>
-      </c>
-      <c r="E607" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>8730000</v>
+      </c>
+      <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>52.17</v>
+        <v>61.01</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J607" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I607" s="6" t="inlineStr"/>
+      <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr"/>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26699,7 +26699,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>23.04.2026 15:30</t>
+          <t>23.04.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 23.04.2026 16:59 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-23.xlsx
+++ b/data/bist_screener_2026-04-23.xlsx
@@ -25824,23 +25824,23 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>28.66</v>
+        <v>251</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0478</v>
+        <v>-0.0346</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>18930000</v>
+        <v>8590</v>
       </c>
       <c r="E584" s="4" t="n">
-        <v>0.2667</v>
+        <v>0.2578</v>
       </c>
       <c r="F584" s="3" t="n">
-        <v>50.42</v>
+        <v>46.72</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
@@ -25848,34 +25848,30 @@
       <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L584" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L584" s="2" t="inlineStr"/>
       <c r="M584" s="2" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>13.89</v>
+        <v>33.9</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.0102</v>
+        <v>-0.0174</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>35540000</v>
+        <v>4590000</v>
       </c>
       <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>54.23</v>
+        <v>54.07</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
@@ -25883,12 +25879,12 @@
       <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25896,21 +25892,21 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>41.38</v>
+        <v>90.84999999999999</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.0222</v>
+        <v>-0.0595</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>10990000</v>
+        <v>14880000</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>60.95</v>
+        <v>61.35</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25918,12 +25914,12 @@
       <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25931,67 +25927,67 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>169</v>
+        <v>81.84</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0236</v>
+        <v>0.0027</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>12070000</v>
+        <v>11800000</v>
       </c>
       <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>60.59</v>
+        <v>45.85</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
       <c r="I587" s="6" t="inlineStr"/>
       <c r="J587" s="6" t="inlineStr"/>
-      <c r="K587" s="6" t="inlineStr">
-        <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+      <c r="K587" s="6" t="inlineStr"/>
+      <c r="L587" s="6" t="inlineStr"/>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>18.99</v>
+        <v>2.74</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0495</v>
+        <v>-0.0108</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>102290000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
-      <c r="F588" s="2" t="inlineStr"/>
+        <v>98340000</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.7119</v>
+      </c>
+      <c r="F588" s="3" t="n">
+        <v>43.27</v>
+      </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J588" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25999,32 +25995,28 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>6.95</v>
+        <v>4.73</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.09970000000000001</v>
+        <v>0.0216</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>75580000</v>
+        <v>62450000</v>
       </c>
       <c r="E589" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.8667</v>
       </c>
       <c r="F589" s="7" t="n">
-        <v>78.58</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J589" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I589" s="6" t="inlineStr"/>
+      <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26032,7 +26024,7 @@
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26040,24 +26032,20 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>4.73</v>
+        <v>103.5</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0216</v>
+        <v>-0.001</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>62450000</v>
-      </c>
-      <c r="E590" s="4" t="n">
-        <v>0.8667</v>
-      </c>
-      <c r="F590" s="3" t="n">
-        <v>77.90000000000001</v>
-      </c>
+        <v>398550</v>
+      </c>
+      <c r="E590" s="2" t="inlineStr"/>
+      <c r="F590" s="2" t="inlineStr"/>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="2" t="inlineStr"/>
@@ -26067,147 +26055,149 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L590" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
-        </is>
-      </c>
+      <c r="L590" s="2" t="inlineStr"/>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>7.59</v>
+        <v>41.38</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.007800000000000001</v>
+        <v>0.0222</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>477650</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>10990000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>39.58</v>
+        <v>60.95</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J591" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I591" s="6" t="inlineStr"/>
+      <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>81.84</v>
+        <v>62.95</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0027</v>
+        <v>-0.0008</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>11800000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>539710</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>45.85</v>
+        <v>56.09</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="2" t="inlineStr"/>
-      <c r="K592" s="2" t="inlineStr"/>
-      <c r="L592" s="2" t="inlineStr"/>
+      <c r="J592" s="4" t="n">
+        <v>0.4139</v>
+      </c>
+      <c r="K592" s="2" t="inlineStr">
+        <is>
+          <t>Teknoloji hizmetleri</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>62.95</v>
+        <v>7.59</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0008</v>
+        <v>-0.007800000000000001</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>539710</v>
+        <v>477650</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>56.09</v>
+        <v>39.58</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
       <c r="J593" s="8" t="n">
-        <v>0.4139</v>
+        <v>-0.4678</v>
       </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>197.4</v>
+        <v>18.99</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.099</v>
+        <v>-0.0495</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>20610000</v>
+        <v>102290000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
-      <c r="F594" s="3" t="n">
-        <v>45.87</v>
-      </c>
+      <c r="F594" s="2" t="inlineStr"/>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
       <c r="I594" s="2" t="inlineStr"/>
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26215,42 +26205,34 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>17.32</v>
+        <v>24.62</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0058</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>12210000</v>
-      </c>
-      <c r="E595" s="8" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>15600000</v>
+      </c>
+      <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>47.99</v>
-      </c>
-      <c r="G595" s="7" t="n">
-        <v>163.71</v>
-      </c>
+        <v>56.05</v>
+      </c>
+      <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J595" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I595" s="6" t="inlineStr"/>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26258,42 +26240,32 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>2.74</v>
+        <v>6.13</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0108</v>
+        <v>0.0016</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>98340000</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>8730000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>43.27</v>
+        <v>61.01</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J596" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I596" s="2" t="inlineStr"/>
+      <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr"/>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
@@ -26336,26 +26308,32 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>2.82</v>
+        <v>6.95</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0537</v>
+        <v>-0.09970000000000001</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>263430000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>75580000</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>52.07</v>
+        <v>78.58</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="I598" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J598" s="4" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26363,7 +26341,7 @@
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26406,40 +26384,34 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>152.1</v>
+        <v>197.4</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0225</v>
+        <v>-0.099</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>2330000</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>20610000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>52.17</v>
+        <v>45.87</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26447,63 +26419,75 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>103.5</v>
+        <v>39.64</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.001</v>
+        <v>0.0195</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>398550</v>
+        <v>12770000</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
-      <c r="F601" s="6" t="inlineStr"/>
+      <c r="F601" s="7" t="n">
+        <v>52.02</v>
+      </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>33.9</v>
+        <v>152.1</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0174</v>
+        <v>-0.0225</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>4590000</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>2330000</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>54.07</v>
+        <v>52.17</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="2" t="inlineStr"/>
-      <c r="J602" s="2" t="inlineStr"/>
+      <c r="I602" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J602" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26511,21 +26495,21 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>39.64</v>
+        <v>2.82</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0195</v>
+        <v>-0.0537</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>12770000</v>
+        <v>263430000</v>
       </c>
       <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>52.02</v>
+        <v>52.07</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26533,12 +26517,12 @@
       <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26546,21 +26530,21 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>90.84999999999999</v>
+        <v>169</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0595</v>
+        <v>0.0236</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>14880000</v>
+        <v>12070000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>61.35</v>
+        <v>60.59</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26573,7 +26557,7 @@
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26581,21 +26565,23 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>24.62</v>
+        <v>28.66</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.004099999999999999</v>
+        <v>-0.0478</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>15600000</v>
-      </c>
-      <c r="E605" s="6" t="inlineStr"/>
+        <v>18930000</v>
+      </c>
+      <c r="E605" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F605" s="7" t="n">
-        <v>56.05</v>
+        <v>50.42</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26603,12 +26589,12 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26616,23 +26602,21 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>251</v>
+        <v>13.89</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0346</v>
+        <v>0.0102</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>8590</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>35540000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>46.72</v>
+        <v>54.23</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26643,38 +26627,54 @@
           <t>İşlenebilen endüstriler</t>
         </is>
       </c>
-      <c r="L606" s="2" t="inlineStr"/>
+      <c r="L606" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>6.13</v>
+        <v>17.32</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0016</v>
+        <v>0.0058</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>8730000</v>
-      </c>
-      <c r="E607" s="6" t="inlineStr"/>
+        <v>12210000</v>
+      </c>
+      <c r="E607" s="8" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F607" s="7" t="n">
-        <v>61.01</v>
-      </c>
-      <c r="G607" s="6" t="inlineStr"/>
+        <v>47.99</v>
+      </c>
+      <c r="G607" s="7" t="n">
+        <v>163.71</v>
+      </c>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="6" t="inlineStr"/>
-      <c r="J607" s="6" t="inlineStr"/>
+      <c r="I607" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J607" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+        </is>
+      </c>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26699,7 +26699,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>23.04.2026 16:30</t>
+          <t>23.04.2026 16:59</t>
         </is>
       </c>
     </row>

</xml_diff>